<commit_message>
Add Edit and Delete functionality to haulage report
</commit_message>
<xml_diff>
--- a/data/field_polygons.xlsx
+++ b/data/field_polygons.xlsx
@@ -1,15 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sibale\Desktop\Flask FarmManagementSystem\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -319,8 +324,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -383,6 +388,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -429,7 +442,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -461,9 +474,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -495,6 +509,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -670,11 +685,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -694,7 +709,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -714,7 +729,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -725,7 +740,7 @@
         <v>55</v>
       </c>
       <c r="D3">
-        <v>9.135</v>
+        <v>9.1349999999999998</v>
       </c>
       <c r="E3" t="s">
         <v>58</v>
@@ -734,7 +749,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -754,7 +769,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -774,7 +789,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -785,7 +800,7 @@
         <v>55</v>
       </c>
       <c r="D6">
-        <v>17.124</v>
+        <v>17.123999999999999</v>
       </c>
       <c r="E6" t="s">
         <v>61</v>
@@ -794,7 +809,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -814,7 +829,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -825,7 +840,7 @@
         <v>55</v>
       </c>
       <c r="D8">
-        <v>23.658</v>
+        <v>23.658000000000001</v>
       </c>
       <c r="E8" t="s">
         <v>63</v>
@@ -834,7 +849,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -854,7 +869,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -874,7 +889,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -894,7 +909,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -905,7 +920,7 @@
         <v>55</v>
       </c>
       <c r="D12">
-        <v>10.646</v>
+        <v>10.646000000000001</v>
       </c>
       <c r="E12" t="s">
         <v>67</v>
@@ -914,7 +929,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -934,7 +949,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -954,7 +969,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -965,7 +980,7 @@
         <v>55</v>
       </c>
       <c r="D15">
-        <v>17.504</v>
+        <v>17.504000000000001</v>
       </c>
       <c r="E15" t="s">
         <v>70</v>
@@ -974,7 +989,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -994,7 +1009,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1005,7 +1020,7 @@
         <v>54</v>
       </c>
       <c r="D17">
-        <v>17.328</v>
+        <v>17.327999999999999</v>
       </c>
       <c r="E17" t="s">
         <v>72</v>
@@ -1014,7 +1029,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -1034,7 +1049,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -1045,7 +1060,7 @@
         <v>54</v>
       </c>
       <c r="D19">
-        <v>7.174</v>
+        <v>7.1740000000000004</v>
       </c>
       <c r="E19" t="s">
         <v>74</v>
@@ -1054,7 +1069,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -1074,7 +1089,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -1094,7 +1109,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -1105,7 +1120,7 @@
         <v>56</v>
       </c>
       <c r="D22">
-        <v>16.079</v>
+        <v>16.079000000000001</v>
       </c>
       <c r="E22" t="s">
         <v>77</v>
@@ -1114,7 +1129,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -1125,7 +1140,7 @@
         <v>56</v>
       </c>
       <c r="D23">
-        <v>16.889</v>
+        <v>16.888999999999999</v>
       </c>
       <c r="E23" t="s">
         <v>78</v>
@@ -1134,7 +1149,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1154,7 +1169,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -1165,7 +1180,7 @@
         <v>56</v>
       </c>
       <c r="D25">
-        <v>19.15</v>
+        <v>19.149999999999999</v>
       </c>
       <c r="E25" t="s">
         <v>80</v>
@@ -1174,7 +1189,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -1185,7 +1200,7 @@
         <v>56</v>
       </c>
       <c r="D26">
-        <v>18.325</v>
+        <v>18.324999999999999</v>
       </c>
       <c r="E26" t="s">
         <v>81</v>
@@ -1194,7 +1209,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -1214,7 +1229,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -1225,7 +1240,7 @@
         <v>56</v>
       </c>
       <c r="D28">
-        <v>8.904</v>
+        <v>8.9039999999999999</v>
       </c>
       <c r="E28" t="s">
         <v>83</v>
@@ -1234,7 +1249,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -1245,7 +1260,7 @@
         <v>56</v>
       </c>
       <c r="D29">
-        <v>21.858</v>
+        <v>21.858000000000001</v>
       </c>
       <c r="E29" t="s">
         <v>84</v>
@@ -1254,7 +1269,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -1265,7 +1280,7 @@
         <v>56</v>
       </c>
       <c r="D30">
-        <v>23.162</v>
+        <v>23.161999999999999</v>
       </c>
       <c r="E30" t="s">
         <v>85</v>
@@ -1274,7 +1289,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -1285,7 +1300,7 @@
         <v>56</v>
       </c>
       <c r="D31">
-        <v>24.107</v>
+        <v>24.106999999999999</v>
       </c>
       <c r="E31" t="s">
         <v>86</v>
@@ -1294,7 +1309,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -1305,7 +1320,7 @@
         <v>56</v>
       </c>
       <c r="D32">
-        <v>25.193</v>
+        <v>25.193000000000001</v>
       </c>
       <c r="E32" t="s">
         <v>87</v>
@@ -1314,7 +1329,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -1325,7 +1340,7 @@
         <v>56</v>
       </c>
       <c r="D33">
-        <v>24.804</v>
+        <v>24.803999999999998</v>
       </c>
       <c r="E33" t="s">
         <v>88</v>
@@ -1334,7 +1349,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -1345,7 +1360,7 @@
         <v>56</v>
       </c>
       <c r="D34">
-        <v>23.147</v>
+        <v>23.146999999999998</v>
       </c>
       <c r="E34" t="s">
         <v>89</v>
@@ -1354,7 +1369,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -1374,7 +1389,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -1385,7 +1400,7 @@
         <v>56</v>
       </c>
       <c r="D36">
-        <v>4.195</v>
+        <v>4.1950000000000003</v>
       </c>
       <c r="E36" t="s">
         <v>91</v>
@@ -1394,7 +1409,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -1405,7 +1420,7 @@
         <v>56</v>
       </c>
       <c r="D37">
-        <v>8.738</v>
+        <v>8.7379999999999995</v>
       </c>
       <c r="E37" t="s">
         <v>92</v>
@@ -1414,7 +1429,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1425,7 +1440,7 @@
         <v>56</v>
       </c>
       <c r="D38">
-        <v>25.047</v>
+        <v>25.047000000000001</v>
       </c>
       <c r="E38" t="s">
         <v>93</v>
@@ -1434,7 +1449,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -1445,7 +1460,7 @@
         <v>56</v>
       </c>
       <c r="D39">
-        <v>21.138</v>
+        <v>21.138000000000002</v>
       </c>
       <c r="E39" t="s">
         <v>94</v>
@@ -1454,7 +1469,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -1465,7 +1480,7 @@
         <v>56</v>
       </c>
       <c r="D40">
-        <v>24.543</v>
+        <v>24.542999999999999</v>
       </c>
       <c r="E40" t="s">
         <v>95</v>
@@ -1474,7 +1489,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1485,7 +1500,7 @@
         <v>56</v>
       </c>
       <c r="D41">
-        <v>12.601</v>
+        <v>12.601000000000001</v>
       </c>
       <c r="E41" t="s">
         <v>96</v>
@@ -1494,7 +1509,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -1505,7 +1520,7 @@
         <v>54</v>
       </c>
       <c r="D42">
-        <v>9.779999999999999</v>
+        <v>9.7799999999999994</v>
       </c>
       <c r="E42" t="s">
         <v>97</v>
@@ -1514,7 +1529,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
Update data files and modules for irrigation sync and GDrive integration
</commit_message>
<xml_diff>
--- a/data/field_polygons.xlsx
+++ b/data/field_polygons.xlsx
@@ -1,20 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sibale\Desktop\Flask FarmManagementSystem\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -324,8 +319,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -388,14 +383,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -442,7 +429,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -474,10 +461,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -509,7 +495,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -685,11 +670,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -709,7 +694,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -729,7 +714,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -740,7 +725,7 @@
         <v>55</v>
       </c>
       <c r="D3">
-        <v>9.1349999999999998</v>
+        <v>9.135</v>
       </c>
       <c r="E3" t="s">
         <v>58</v>
@@ -749,7 +734,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -769,7 +754,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -789,7 +774,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -800,7 +785,7 @@
         <v>55</v>
       </c>
       <c r="D6">
-        <v>17.123999999999999</v>
+        <v>17.124</v>
       </c>
       <c r="E6" t="s">
         <v>61</v>
@@ -809,7 +794,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -829,7 +814,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -840,7 +825,7 @@
         <v>55</v>
       </c>
       <c r="D8">
-        <v>23.658000000000001</v>
+        <v>23.658</v>
       </c>
       <c r="E8" t="s">
         <v>63</v>
@@ -849,7 +834,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -869,7 +854,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -889,7 +874,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -909,7 +894,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -920,7 +905,7 @@
         <v>55</v>
       </c>
       <c r="D12">
-        <v>10.646000000000001</v>
+        <v>10.646</v>
       </c>
       <c r="E12" t="s">
         <v>67</v>
@@ -929,7 +914,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -949,7 +934,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -969,7 +954,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -980,7 +965,7 @@
         <v>55</v>
       </c>
       <c r="D15">
-        <v>17.504000000000001</v>
+        <v>17.504</v>
       </c>
       <c r="E15" t="s">
         <v>70</v>
@@ -989,7 +974,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -1009,7 +994,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1020,7 +1005,7 @@
         <v>54</v>
       </c>
       <c r="D17">
-        <v>17.327999999999999</v>
+        <v>17.328</v>
       </c>
       <c r="E17" t="s">
         <v>72</v>
@@ -1029,7 +1014,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -1049,7 +1034,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -1060,7 +1045,7 @@
         <v>54</v>
       </c>
       <c r="D19">
-        <v>7.1740000000000004</v>
+        <v>7.174</v>
       </c>
       <c r="E19" t="s">
         <v>74</v>
@@ -1069,7 +1054,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -1089,7 +1074,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -1109,7 +1094,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -1120,7 +1105,7 @@
         <v>56</v>
       </c>
       <c r="D22">
-        <v>16.079000000000001</v>
+        <v>16.079</v>
       </c>
       <c r="E22" t="s">
         <v>77</v>
@@ -1129,7 +1114,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -1140,7 +1125,7 @@
         <v>56</v>
       </c>
       <c r="D23">
-        <v>16.888999999999999</v>
+        <v>16.889</v>
       </c>
       <c r="E23" t="s">
         <v>78</v>
@@ -1149,7 +1134,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1169,7 +1154,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -1180,7 +1165,7 @@
         <v>56</v>
       </c>
       <c r="D25">
-        <v>19.149999999999999</v>
+        <v>19.15</v>
       </c>
       <c r="E25" t="s">
         <v>80</v>
@@ -1189,7 +1174,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -1200,7 +1185,7 @@
         <v>56</v>
       </c>
       <c r="D26">
-        <v>18.324999999999999</v>
+        <v>18.325</v>
       </c>
       <c r="E26" t="s">
         <v>81</v>
@@ -1209,7 +1194,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -1229,7 +1214,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -1240,7 +1225,7 @@
         <v>56</v>
       </c>
       <c r="D28">
-        <v>8.9039999999999999</v>
+        <v>8.904</v>
       </c>
       <c r="E28" t="s">
         <v>83</v>
@@ -1249,7 +1234,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -1260,7 +1245,7 @@
         <v>56</v>
       </c>
       <c r="D29">
-        <v>21.858000000000001</v>
+        <v>21.858</v>
       </c>
       <c r="E29" t="s">
         <v>84</v>
@@ -1269,7 +1254,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -1280,7 +1265,7 @@
         <v>56</v>
       </c>
       <c r="D30">
-        <v>23.161999999999999</v>
+        <v>23.162</v>
       </c>
       <c r="E30" t="s">
         <v>85</v>
@@ -1289,7 +1274,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -1300,7 +1285,7 @@
         <v>56</v>
       </c>
       <c r="D31">
-        <v>24.106999999999999</v>
+        <v>24.107</v>
       </c>
       <c r="E31" t="s">
         <v>86</v>
@@ -1309,7 +1294,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -1320,7 +1305,7 @@
         <v>56</v>
       </c>
       <c r="D32">
-        <v>25.193000000000001</v>
+        <v>25.193</v>
       </c>
       <c r="E32" t="s">
         <v>87</v>
@@ -1329,7 +1314,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -1340,7 +1325,7 @@
         <v>56</v>
       </c>
       <c r="D33">
-        <v>24.803999999999998</v>
+        <v>24.804</v>
       </c>
       <c r="E33" t="s">
         <v>88</v>
@@ -1349,7 +1334,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -1360,7 +1345,7 @@
         <v>56</v>
       </c>
       <c r="D34">
-        <v>23.146999999999998</v>
+        <v>23.147</v>
       </c>
       <c r="E34" t="s">
         <v>89</v>
@@ -1369,7 +1354,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -1389,7 +1374,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -1400,7 +1385,7 @@
         <v>56</v>
       </c>
       <c r="D36">
-        <v>4.1950000000000003</v>
+        <v>4.195</v>
       </c>
       <c r="E36" t="s">
         <v>91</v>
@@ -1409,7 +1394,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -1420,7 +1405,7 @@
         <v>56</v>
       </c>
       <c r="D37">
-        <v>8.7379999999999995</v>
+        <v>8.738</v>
       </c>
       <c r="E37" t="s">
         <v>92</v>
@@ -1429,7 +1414,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1440,7 +1425,7 @@
         <v>56</v>
       </c>
       <c r="D38">
-        <v>25.047000000000001</v>
+        <v>25.047</v>
       </c>
       <c r="E38" t="s">
         <v>93</v>
@@ -1449,7 +1434,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -1460,7 +1445,7 @@
         <v>56</v>
       </c>
       <c r="D39">
-        <v>21.138000000000002</v>
+        <v>21.138</v>
       </c>
       <c r="E39" t="s">
         <v>94</v>
@@ -1469,7 +1454,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -1480,7 +1465,7 @@
         <v>56</v>
       </c>
       <c r="D40">
-        <v>24.542999999999999</v>
+        <v>24.543</v>
       </c>
       <c r="E40" t="s">
         <v>95</v>
@@ -1489,7 +1474,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1500,7 +1485,7 @@
         <v>56</v>
       </c>
       <c r="D41">
-        <v>12.601000000000001</v>
+        <v>12.601</v>
       </c>
       <c r="E41" t="s">
         <v>96</v>
@@ -1509,7 +1494,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -1520,7 +1505,7 @@
         <v>54</v>
       </c>
       <c r="D42">
-        <v>9.7799999999999994</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="E42" t="s">
         <v>97</v>
@@ -1529,7 +1514,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6">
       <c r="A43" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
🚀 Full update: GIS stress level auto update, inventory, harvesting program, and more
</commit_message>
<xml_diff>
--- a/data/field_polygons.xlsx
+++ b/data/field_polygons.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="100">
-  <si>
-    <t>Field Name</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="102">
+  <si>
+    <t>Field</t>
   </si>
   <si>
     <t>Crop</t>
@@ -311,6 +311,12 @@
   </si>
   <si>
     <t>{"type": "FeatureCollection", "features": [{"type": "Feature", "properties": {}, "geometry": {"type": "Polygon", "coordinates": [[[34.150497, -12.555148], [34.148115, -12.556498], [34.148689, -12.557086], [34.14952, -12.557955], [34.150454, -12.558865], [34.150556, -12.558892], [34.150743, -12.558682], [34.151672, -12.558169], [34.152605, -12.557698], [34.15297, -12.557536], [34.151757, -12.556332], [34.150497, -12.555148]]]}}]}</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>Moderate</t>
   </si>
   <si>
     <t>Low</t>
@@ -811,7 +817,7 @@
         <v>62</v>
       </c>
       <c r="F7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -991,7 +997,7 @@
         <v>71</v>
       </c>
       <c r="F16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1011,7 +1017,7 @@
         <v>72</v>
       </c>
       <c r="F17" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1031,7 +1037,7 @@
         <v>73</v>
       </c>
       <c r="F18" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:6">

</xml_diff>